<commit_message>
chore: refresh WISE.L data, valuation anchor and dashboard
Data fixes through make fix: FY take rates added (0.63-0.52%); FY active
customers switched to Wise's customers-served-in-the-year figure (18.9m FY2026)
instead of the Q4 quarterly count; pre-FY2025 volumes and balances converted
from GBP at the per-year revenue factor; volume, holdings, balances and assets
under custody promoted. Re-anchored at 874.0p / GBPUSD 1.3222 (weighted IV
1,033p). Valuation philosophy rewritten to match the 22-Sep model. Analysis
refreshed to 2026-10-06 (US class actions, NBB order, AGM). Dashboard gains
volume, holdings, interest-income, yield and revenue-per-customer charts, a
key-signals box and Wise-specific help text; the float-inflated OCF chart is
gone. Dropped a byte-identical duplicate of the FY2026 20-F text.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/WISE.L/Reports/WISE.L_DCF_Model.xlsx
+++ b/research/WISE.L/Reports/WISE.L_DCF_Model.xlsx
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Built at</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-22T08:28:18Z</t>
+    <t xml:space="preserve">2026-10-05T20:30:52Z</t>
   </si>
   <si>
     <t xml:space="preserve">Drivers file</t>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Methodology</t>
   </si>
   <si>
-    <t xml:space="preserve">Wise is modeled as a decelerating high-growth fintech using a 10-year component-built owner-FCF model, not a flat-margin extrapolation of the FY2026 heavy-investment year. Net revenue CAGR (29.7% trailing 3yr) is the growth driver, not equity CAGR (41.0%, inflated by retained-earnings/FX-translation compounding) or reported FCF (which swings 12.8%-31.8% margin on net revenue with no clean trend due to working-capital/tax timing). Owner FCF is built bottom-up each year: adjusted EBITDA margin ramps from the FY2026 trough (28.5%, post the deliberate compliance/tech/marketing reinvestment step-up) toward a mature 36% (base case) -- materially below the pre-reset FY2024/25 peak of ~42.5%/38.7%, honoring the mandate that Servicing+G&amp;A opex near 30-31% of net revenue is now a permanent structural floor, not a temporary spike. SBC is deducted at its actual (small, ~3.8% of revenue, declining) level -- Wise's near-nil-strike option program plus a buyback ($473.4m FY2026) running ~5x SBC means uncovered dilution is zero and the share count stays flat, the opposite dynamic to DUOL. Working capital is modeled as a net DRAG scaling with revenue growth (not a subscription-style deferred-revenue tailwind), matching Wise's actual multi-year pattern. Net corporate cash (+$1,873.7m, replacing a near-zero net-debt assumption in the prior model) is added to enterprise value, with the offsetting corporate interest income ($63.0m) stripped from FCF to avoid double-counting. WACC (11.5% base) explicitly stacks a 200bp regulatory risk premium across the OCC charter denial, the Belgian criminal AML investigation into Wise Europe SA, and the pattern of repeat AML findings across three jurisdictions in twelve months, plus a 25bp governance premium for the CEO's extended supervoting control -- on top of a ~9.0% base cost of capital for a large, profitable, net-cash global payments platform. The historical-multiple sanity check passes without requiring any fix: base-case implied multiples sit below Wise's own FY2024-26 trading range and assume no multiple expansion (implied exit multiples of 9.3-14.8x vs today's trailing 21.1x EV/owner-FCF). || UPDATED 2026-08-28: the terminal adj-EBITDA margin was cut from 36% to 30% and flattened from Y7 after comparison against two independently built external workbooks, both of which put the mature margin materially lower (27.5% and 30.0%). Combined with a +11.6% USD price move, WISE goes from ~13% base-case upside to ~12% OVERVALUED, and the probability-weighted case from +16.6% to -8.5%. The honest read is that the prior model's headline upside rested on a terminal margin above the company's own pre-investment peak. || 2026-09-22 revision: base margins constrained to management's guided band (terminal EBIT ~22.4% ex corporate interest), one 9.5% USD discount rate for all scenarios with the regulatory risk carried in the bear flows and house 15/50/35 weights (no triple charge), working capital at the three-year actual drag, and shares and cash on the same balance-sheet date. Base moves 876p -&gt; ~920p; the scenario spread narrows and entry prices fall ~100p.</t>
+    <t xml:space="preserve">Wise is valued with a 10-year component-built owner-FCF DCF in USD; the per-share results are converted to pence at the spot rate (GBPUSD 1.3222 on 5-Oct-2026) so they compare directly with the LSE price. Revenue is the driver: base growth fades from 17% to 5.5% over ten years (bull 21% to 7%, bear 11% then 4-7%), consistent with the guided mid-teens-to-20% net revenue growth for FY2027. Margins are held inside management's guidance rather than the old peak: base adjusted EBITDA margin goes from 28.5% to 26% by year 7, which leaves a terminal EBIT of about 22% -- the top of the 20-25% income-before-tax band once the ~2.5pp of corporate interest it includes is removed. The FY2024-25 margins of 35-40% are treated as gone for good because compliance and servicing spend has reset higher. Owner FCF deducts SBC (~3.7% of revenue), lease costs and interest earned on Wise's own cash; working capital is a drag of 25% of each year's revenue increase (the three-year actual average). The $473m share purchase in FY2026 was the Employee Share Trust covering awards, not a capital return; the up-to-GBP405m buyback that started in July 2026 is not modelled. One 9.5% discount rate is used for every scenario, and the regulatory risk (Belgian criminal AML case, OCC charter denial, US consent order, securities class actions) is carried in the bear case's cash flows and its 15% weight rather than charged again through the rate. Net corporate cash of $1.87bn is added to equity value against 1,024m fully diluted shares at the same 31-Mar-2026 date. Result at 874p: bear 533p, base 930p, bull 1,393p, probability-weighted (15/50/35) 1,033p, about 18% above the price; a 15% annual return needs an entry near 535p on the base case (577p probability-weighted). Known limit: the engine uses one equity bridge for all scenarios, so a large AML fine in the bear case is described here but not subtracted (bear is roughly 45p too high).</t>
   </si>
   <si>
     <t xml:space="preserve">WACC rationale</t>
@@ -364,19 +364,19 @@
     <t xml:space="preserve">ShareRepurchases</t>
   </si>
   <si>
-    <t xml:space="preserve">ActiveCustomers_k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CrossBorderVolume_bn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CustomerHoldings_bn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TakeRate_pct</t>
-  </si>
-  <si>
     <t xml:space="preserve">ActiveCustomers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AssetsUnderCustody</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CrossBorderVolume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CustomerBalances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CustomerHoldings</t>
   </si>
   <si>
     <t xml:space="preserve">TakeRate</t>
@@ -1016,7 +1016,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>863.8</v>
+        <v>874</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1257,7 +1257,7 @@
         <v>53</v>
       </c>
       <c r="B11" s="0" t="n">
-        <v>863.8</v>
+        <v>874</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1265,7 +1265,7 @@
         <v>54</v>
       </c>
       <c r="B12" s="0" t="n">
-        <v>527.54</v>
+        <v>533.12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1273,7 +1273,7 @@
         <v>55</v>
       </c>
       <c r="B13" s="0" t="n">
-        <v>920.07</v>
+        <v>929.82</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1281,7 +1281,7 @@
         <v>56</v>
       </c>
       <c r="B14" s="0" t="n">
-        <v>1378.6</v>
+        <v>1393.2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1289,7 +1289,7 @@
         <v>57</v>
       </c>
       <c r="B15" s="0" t="n">
-        <v>1021.68</v>
+        <v>1032.5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1692,10 +1692,16 @@
         <v>0</v>
       </c>
       <c r="AI3" s="0" t="n">
-        <v>4588</v>
-      </c>
-      <c r="AM3" s="0" t="n">
-        <v>4588</v>
+        <v>7400</v>
+      </c>
+      <c r="AK3" s="0" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="AL3" s="0" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="AN3" s="0" t="n">
+        <v>0.63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1787,10 +1793,22 @@
         <v>12</v>
       </c>
       <c r="AI4" s="0" t="n">
-        <v>6125</v>
+        <v>9962.7</v>
+      </c>
+      <c r="AJ4" s="0" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="AK4" s="0" t="n">
+        <v>124.35</v>
+      </c>
+      <c r="AL4" s="0" t="n">
+        <v>12.73</v>
       </c>
       <c r="AM4" s="0" t="n">
-        <v>6125</v>
+        <v>13.33</v>
+      </c>
+      <c r="AN4" s="0" t="n">
+        <v>0.65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1882,10 +1900,22 @@
         <v>86.2</v>
       </c>
       <c r="AI5" s="0" t="n">
-        <v>7911</v>
+        <v>12838.2</v>
+      </c>
+      <c r="AJ5" s="0" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="AK5" s="0" t="n">
+        <v>149.03</v>
+      </c>
+      <c r="AL5" s="0" t="n">
+        <v>16.73</v>
       </c>
       <c r="AM5" s="0" t="n">
-        <v>7911</v>
+        <v>20.37</v>
+      </c>
+      <c r="AN5" s="0" t="n">
+        <v>0.67</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1977,16 +2007,22 @@
         <v>92.5</v>
       </c>
       <c r="AI6" s="0" t="n">
-        <v>9290</v>
+        <v>15566.1</v>
       </c>
       <c r="AJ6" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="AK6" s="0" t="n">
         <v>185.2</v>
       </c>
-      <c r="AK6" s="0" t="n">
+      <c r="AL6" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="AM6" s="0" t="n">
         <v>27.8</v>
       </c>
-      <c r="AM6" s="0" t="n">
-        <v>9290</v>
+      <c r="AN6" s="0" t="n">
+        <v>0.58</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2078,16 +2114,22 @@
         <v>473.4</v>
       </c>
       <c r="AI7" s="0" t="n">
-        <v>11290</v>
+        <v>18900</v>
       </c>
       <c r="AJ7" s="0" t="n">
-        <v>243.6</v>
+        <v>9</v>
       </c>
       <c r="AK7" s="0" t="n">
+        <v>243.5</v>
+      </c>
+      <c r="AL7" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="AM7" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="AM7" s="0" t="n">
-        <v>11290</v>
+      <c r="AN7" s="0" t="n">
+        <v>0.52</v>
       </c>
     </row>
   </sheetData>
@@ -2125,7 +2167,7 @@
         <v>120</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>863.8</v>
+        <v>874</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2189,7 +2231,7 @@
         <v>129</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>74.8391</v>
+        <v>75.6315</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4233,7 +4275,7 @@
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>527.536004993016</v>
+        <v>533.121581654901</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4242,7 +4284,7 @@
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>-0.389284550830035</v>
+        <v>-0.390021073621395</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4269,7 +4311,7 @@
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>653.416102257211</v>
+        <v>660.334503459639</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4296,7 +4338,7 @@
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>356.033546264205</v>
+        <v>359.80324662217</v>
       </c>
     </row>
   </sheetData>
@@ -5380,7 +5422,7 @@
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>920.074670571902</v>
+        <v>929.816465555556</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5389,7 +5431,7 @@
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>0.0651478010788404</v>
+        <v>0.0638632329010942</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5416,7 +5458,7 @@
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1087.90104699711</v>
+        <v>1099.41979574797</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5443,7 +5485,7 @@
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>528.988656836476</v>
+        <v>534.589614246135</v>
       </c>
     </row>
   </sheetData>
@@ -6527,7 +6569,7 @@
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1378.60090477275</v>
+        <v>1393.19759763707</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6536,7 +6578,7 @@
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>0.595972337083527</v>
+        <v>0.594047594550421</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6563,7 +6605,7 @@
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1559.45686342592</v>
+        <v>1575.96846790244</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6590,7 +6632,7 @@
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>723.322192257219</v>
+        <v>730.980762511867</v>
       </c>
     </row>
   </sheetData>
@@ -6646,11 +6688,11 @@
       </c>
       <c r="B4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$38</f>
-        <v>527.536004993016</v>
+        <v>533.121581654901</v>
       </c>
       <c r="C4" s="0" t="n">
         <f aca="false">B4/Assumptions!$B$2-1</f>
-        <v>-0.389284550830035</v>
+        <v>-0.390021073621395</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">Assumptions!$B$24</f>
@@ -6658,11 +6700,11 @@
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$43</f>
-        <v>653.416102257211</v>
+        <v>660.334503459639</v>
       </c>
       <c r="F4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$47</f>
-        <v>356.033546264205</v>
+        <v>359.80324662217</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6671,11 +6713,11 @@
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">DCF_Base!$B$38</f>
-        <v>920.074670571902</v>
+        <v>929.816465555556</v>
       </c>
       <c r="C5" s="0" t="n">
         <f aca="false">B5/Assumptions!$B$2-1</f>
-        <v>0.0651478010788404</v>
+        <v>0.0638632329010942</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">Assumptions!$B$38</f>
@@ -6683,11 +6725,11 @@
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">DCF_Base!$B$43</f>
-        <v>1087.90104699711</v>
+        <v>1099.41979574797</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">DCF_Base!$B$47</f>
-        <v>528.988656836476</v>
+        <v>534.589614246135</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6696,11 +6738,11 @@
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$38</f>
-        <v>1378.60090477275</v>
+        <v>1393.19759763707</v>
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">B6/Assumptions!$B$2-1</f>
-        <v>0.595972337083527</v>
+        <v>0.594047594550421</v>
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">Assumptions!$B$52</f>
@@ -6708,11 +6750,11 @@
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$43</f>
-        <v>1559.45686342592</v>
+        <v>1575.96846790244</v>
       </c>
       <c r="F6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$47</f>
-        <v>723.322192257219</v>
+        <v>730.980762511867</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6721,7 +6763,7 @@
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">SUMPRODUCT(B4:B6,D4:D6)</f>
-        <v>1021.67805270537</v>
+        <v>1032.49562919899</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6730,7 +6772,7 @@
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">SUMPRODUCT(E4:E6,D4:D6)</f>
-        <v>1187.77284103621</v>
+        <v>1200.34903715879</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6739,7 +6781,7 @@
       </c>
       <c r="B10" s="0" t="n">
         <f aca="false">1-Assumptions!$B$2/B8</f>
-        <v>0.154528182618107</v>
+        <v>0.153507312492885</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6748,7 +6790,7 @@
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">IF(ABS(B9-B8)&gt;0.01*ABS(B8),(Assumptions!$B$2-B8)/(B9-B8)*100,"n/a")</f>
-        <v>-95.0529840773147</v>
+        <v>-94.4250290330398</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6757,7 +6799,7 @@
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">SUMPRODUCT(F4:F6,D4:D6)</f>
-        <v>571.062127647895</v>
+        <v>577.108560995546</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6774,7 +6816,7 @@
       </c>
       <c r="B15" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$15/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$15&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$15-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$15/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>992.302720834185</v>
+        <v>1002.80926989729</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>9</v>
@@ -6786,7 +6828,7 @@
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$16/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$16&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$16-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$16/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>920.074670571902</v>
+        <v>929.816465555556</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>9.5</v>
@@ -6798,7 +6840,7 @@
       </c>
       <c r="B17" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$17/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$17&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$17-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$17/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>858.346069284236</v>
+        <v>867.434278860525</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>10</v>
@@ -6810,7 +6852,7 @@
       </c>
       <c r="B18" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$18/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$18&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$18-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$18/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>758.488657111838</v>
+        <v>766.519571592309</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>11</v>
@@ -6822,7 +6864,7 @@
       </c>
       <c r="B19" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$19/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$19&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$19-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$19/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>681.32379212449</v>
+        <v>688.537681293113</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>12</v>
@@ -6834,7 +6876,7 @@
       </c>
       <c r="B20" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$20/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$20&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$20-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$20/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>528.988656836476</v>
+        <v>534.589614246135</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>15</v>
@@ -6868,23 +6910,23 @@
       </c>
       <c r="B24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$24-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1148.883785758</v>
+        <v>1161.04822268782</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$24-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1201.86689287499</v>
+        <v>1214.59231749814</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$24-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1201.86689287499</v>
+        <v>1214.59231749814</v>
       </c>
       <c r="E24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$24-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1201.86689287499</v>
+        <v>1214.59231749814</v>
       </c>
       <c r="F24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$24-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1201.86689287499</v>
+        <v>1214.59231749814</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6893,23 +6935,23 @@
       </c>
       <c r="B25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$25-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>977.128336565002</v>
+        <v>987.474218515668</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$25-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1023.31669441882</v>
+        <v>1034.15162092993</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$25-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1077.90293551879</v>
+        <v>1089.31582378315</v>
       </c>
       <c r="E25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$25-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1120.16325120909</v>
+        <v>1132.02359373402</v>
       </c>
       <c r="F25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$25-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1120.16325120909</v>
+        <v>1132.02359373402</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6918,23 +6960,23 @@
       </c>
       <c r="B26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$26-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>852.030162972678</v>
+        <v>861.051499428348</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$26-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>883.622255786603</v>
+        <v>892.978090844552</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$26-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>920.074670571902</v>
+        <v>929.816465555556</v>
       </c>
       <c r="E26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$26-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>962.602487821418</v>
+        <v>972.794569385061</v>
       </c>
       <c r="F26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$26-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>1012.86263547994</v>
+        <v>1023.58687391084</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6943,23 +6985,23 @@
       </c>
       <c r="B27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$27-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>757.064375824779</v>
+        <v>765.080209946295</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$27-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>779.539151089969</v>
+        <v>787.792949215864</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$27-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>805.010563057184</v>
+        <v>813.534053721376</v>
       </c>
       <c r="E27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$27-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>834.120748162573</v>
+        <v>842.952458870532</v>
       </c>
       <c r="F27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$27-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>867.709423284176</v>
+        <v>876.896772504175</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6968,23 +7010,23 @@
       </c>
       <c r="B28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$28-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>682.668484758123</v>
+        <v>689.8966115972</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$28-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>699.151051821107</v>
+        <v>706.553696875137</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$28-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>717.572744420913</v>
+        <v>725.170439244597</v>
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$28-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>738.297148595695</v>
+        <v>746.114274410239</v>
       </c>
       <c r="F28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$28-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>761.784806660447</v>
+        <v>769.8506209313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>